<commit_message>
fix bug in constraints, run vol match tests
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/Scripts/Case Studies/1. Portfolio Analysis/Simple Portfolio Report_new_pe.xlsx
+++ b/epsilon-phi-core/src/Scripts/Case Studies/1. Portfolio Analysis/Simple Portfolio Report_new_pe.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/Scripts/Case Studies/1. Portfolio Analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/repo/epsilon-psi/epsilon-phi-core/src/Scripts/Case Studies/1. Portfolio Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE9C429-B145-EF48-BA96-9EB80FE03BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F469C6C1-D1F0-284B-8ECD-3F07464E8F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2200" yWindow="1240" windowWidth="49600" windowHeight="24840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19040" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="portfolios" sheetId="1" r:id="rId1"/>
@@ -875,13 +875,10 @@
     <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -889,18 +886,21 @@
     <xf numFmtId="2" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -7838,7 +7838,7 @@
                   <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -22377,24 +22377,24 @@
   <sheetData>
     <row r="1" spans="1:5" ht="41" customHeight="1">
       <c r="A1" s="42"/>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="67" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="63"/>
-      <c r="D1" s="71" t="s">
+      <c r="D1" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="72"/>
+      <c r="E1" s="69"/>
     </row>
     <row r="2" spans="1:5" ht="16" customHeight="1">
       <c r="A2" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="64">
+      <c r="B2" s="62">
         <v>0.5</v>
       </c>
       <c r="C2" s="63"/>
-      <c r="D2" s="64">
+      <c r="D2" s="62">
         <v>0.36</v>
       </c>
       <c r="E2" s="63"/>
@@ -22403,11 +22403,11 @@
       <c r="A3" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="62" t="s">
         <v>150</v>
       </c>
       <c r="C3" s="63"/>
-      <c r="D3" s="64">
+      <c r="D3" s="62">
         <v>4.4999999999999998E-2</v>
       </c>
       <c r="E3" s="63"/>
@@ -22416,11 +22416,11 @@
       <c r="A4" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="64">
+      <c r="B4" s="62">
         <v>0.5</v>
       </c>
       <c r="C4" s="63"/>
-      <c r="D4" s="64">
+      <c r="D4" s="62">
         <v>0.35499999999999998</v>
       </c>
       <c r="E4" s="63"/>
@@ -22429,11 +22429,11 @@
       <c r="A5" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="64" t="s">
+      <c r="B5" s="62" t="s">
         <v>150</v>
       </c>
       <c r="C5" s="63"/>
-      <c r="D5" s="64">
+      <c r="D5" s="62">
         <v>4.5000000000000012E-2</v>
       </c>
       <c r="E5" s="63"/>
@@ -22442,11 +22442,11 @@
       <c r="A6" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="64" t="s">
+      <c r="B6" s="62" t="s">
         <v>150</v>
       </c>
       <c r="C6" s="63"/>
-      <c r="D6" s="64">
+      <c r="D6" s="62">
         <v>0.12</v>
       </c>
       <c r="E6" s="63"/>
@@ -22455,11 +22455,11 @@
       <c r="A7" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="64" t="s">
+      <c r="B7" s="62" t="s">
         <v>150</v>
       </c>
       <c r="C7" s="63"/>
-      <c r="D7" s="64">
+      <c r="D7" s="62">
         <v>7.5000000000000011E-2</v>
       </c>
       <c r="E7" s="63"/>
@@ -22468,24 +22468,24 @@
       <c r="A8" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="65">
+      <c r="B8" s="64">
         <v>5.3832602562404443E-2</v>
       </c>
-      <c r="C8" s="66"/>
-      <c r="D8" s="65">
+      <c r="C8" s="65"/>
+      <c r="D8" s="64">
         <v>6.4431104932666197E-2</v>
       </c>
-      <c r="E8" s="66"/>
+      <c r="E8" s="65"/>
     </row>
     <row r="9" spans="1:5" ht="16" customHeight="1">
       <c r="A9" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="67">
+      <c r="B9" s="66">
         <v>0.39013325979698232</v>
       </c>
       <c r="C9" s="63"/>
-      <c r="D9" s="67">
+      <c r="D9" s="66">
         <v>0.52364381017028427</v>
       </c>
       <c r="E9" s="63"/>
@@ -22494,11 +22494,11 @@
       <c r="A10" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="64">
+      <c r="B10" s="62">
         <v>7.3904497600149111E-2</v>
       </c>
       <c r="C10" s="63"/>
-      <c r="D10" s="64">
+      <c r="D10" s="62">
         <v>7.5095139422881152E-2</v>
       </c>
       <c r="E10" s="63"/>
@@ -22936,6 +22936,18 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:E6"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="B7:C7"/>
@@ -22944,18 +22956,6 @@
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D9:E9"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="B13:E21">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
@@ -22985,27 +22985,27 @@
   <sheetData>
     <row r="1" spans="1:10" ht="24" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="68" t="s">
+      <c r="B1" s="70" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
       <c r="H1" s="3"/>
-      <c r="I1" s="68" t="s">
+      <c r="I1" s="70" t="s">
         <v>54</v>
       </c>
-      <c r="J1" s="69"/>
+      <c r="J1" s="71"/>
     </row>
     <row r="2" spans="1:10" ht="49" customHeight="1">
       <c r="A2" s="4"/>
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="72" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
       <c r="E2" s="2" t="s">
         <v>33</v>
       </c>

</xml_diff>

<commit_message>
code refactoring and case study additions
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/Scripts/Case Studies/1. Portfolio Analysis/Simple Portfolio Report_new_pe.xlsx
+++ b/epsilon-phi-core/src/Scripts/Case Studies/1. Portfolio Analysis/Simple Portfolio Report_new_pe.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/repo/epsilon-psi/epsilon-phi-core/src/Scripts/Case Studies/1. Portfolio Analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/Scripts/Case Studies/1. Portfolio Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB2D1C3-6880-DC48-8FC8-04065BF04204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061DF6AC-6E24-2742-8C00-96F375277F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1196,6 +1196,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1208,16 +1218,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -22051,7 +22051,9 @@
         <f>SUM(C3:C8)</f>
         <v>3.9323104932666136E-2</v>
       </c>
-      <c r="D2" s="40"/>
+      <c r="D2" s="42">
+        <v>2.23946383044141E-2</v>
+      </c>
       <c r="E2" s="40"/>
       <c r="F2" s="40"/>
       <c r="G2" s="40"/>
@@ -22073,7 +22075,9 @@
       <c r="C3" s="42">
         <v>7.0898094817600603E-4</v>
       </c>
-      <c r="D3" s="40"/>
+      <c r="D3" s="42">
+        <v>5.1102386495189001E-3</v>
+      </c>
       <c r="E3" s="40"/>
       <c r="F3" s="40"/>
       <c r="G3" s="40"/>
@@ -22095,7 +22099,9 @@
       <c r="C4" s="42">
         <v>-7.31425731588811E-5</v>
       </c>
-      <c r="D4" s="40"/>
+      <c r="D4" s="42">
+        <v>1.4935013698618501E-4</v>
+      </c>
       <c r="E4" s="40"/>
       <c r="F4" s="40"/>
       <c r="G4" s="40"/>
@@ -22117,7 +22123,9 @@
       <c r="C5" s="42">
         <v>5.2595580514326603E-3</v>
       </c>
-      <c r="D5" s="40"/>
+      <c r="D5" s="42">
+        <v>2.4458062675070699E-4</v>
+      </c>
       <c r="E5" s="40"/>
       <c r="F5" s="40"/>
       <c r="G5" s="40"/>
@@ -22139,7 +22147,9 @@
       <c r="C6" s="42">
         <v>3.2283957050202399E-3</v>
       </c>
-      <c r="D6" s="40"/>
+      <c r="D6" s="42">
+        <v>2.52168605647219E-4</v>
+      </c>
       <c r="E6" s="40"/>
       <c r="F6" s="40"/>
       <c r="G6" s="40"/>
@@ -22161,7 +22171,9 @@
       <c r="C7" s="42">
         <v>5.9454343476038098E-3</v>
       </c>
-      <c r="D7" s="40"/>
+      <c r="D7" s="42">
+        <v>6.8162623908724399E-4</v>
+      </c>
       <c r="E7" s="40"/>
       <c r="F7" s="40"/>
       <c r="G7" s="40"/>
@@ -22246,7 +22258,9 @@
     <row r="12" spans="1:14">
       <c r="A12" s="40"/>
       <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
+      <c r="C12" s="40">
+        <v>0</v>
+      </c>
       <c r="D12" s="40"/>
       <c r="E12" s="40"/>
       <c r="F12" s="40"/>
@@ -22261,8 +22275,12 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="40"/>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
+      <c r="B13" s="40">
+        <v>0</v>
+      </c>
+      <c r="C13" s="40">
+        <v>2.23946383044141E-2</v>
+      </c>
       <c r="D13" s="40"/>
       <c r="E13" s="40"/>
       <c r="F13" s="40"/>
@@ -22277,8 +22295,12 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="40"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
+      <c r="B14" s="40">
+        <v>1</v>
+      </c>
+      <c r="C14" s="40">
+        <v>5.1102386495189001E-3</v>
+      </c>
       <c r="D14" s="40"/>
       <c r="E14" s="40"/>
       <c r="F14" s="40"/>
@@ -22293,8 +22315,12 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="40"/>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
+      <c r="B15" s="40">
+        <v>2</v>
+      </c>
+      <c r="C15" s="40">
+        <v>1.4935013698618501E-4</v>
+      </c>
       <c r="D15" s="40"/>
       <c r="E15" s="40"/>
       <c r="F15" s="40"/>
@@ -22309,8 +22335,12 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="40"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
+      <c r="B16" s="40">
+        <v>3</v>
+      </c>
+      <c r="C16" s="40">
+        <v>2.4458062675070699E-4</v>
+      </c>
       <c r="D16" s="40"/>
       <c r="E16" s="40"/>
       <c r="F16" s="40"/>
@@ -22325,8 +22355,12 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="40"/>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
+      <c r="B17" s="40">
+        <v>4</v>
+      </c>
+      <c r="C17" s="40">
+        <v>2.52168605647219E-4</v>
+      </c>
       <c r="D17" s="40"/>
       <c r="E17" s="40"/>
       <c r="F17" s="40"/>
@@ -22341,8 +22375,12 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="40"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
+      <c r="B18" s="40">
+        <v>5</v>
+      </c>
+      <c r="C18" s="40">
+        <v>6.8162623908724399E-4</v>
+      </c>
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
       <c r="F18" s="40"/>
@@ -22899,131 +22937,131 @@
   <sheetData>
     <row r="1" spans="1:5" ht="41" customHeight="1">
       <c r="A1" s="66"/>
-      <c r="B1" s="97" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="98"/>
-      <c r="D1" s="99" t="s">
+      <c r="B1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="91"/>
+      <c r="D1" s="92" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="100"/>
+      <c r="E1" s="93"/>
     </row>
     <row r="2" spans="1:5" ht="16" customHeight="1">
       <c r="A2" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="90">
+      <c r="B2" s="94">
         <v>0.5</v>
       </c>
-      <c r="C2" s="91"/>
-      <c r="D2" s="90">
+      <c r="C2" s="95"/>
+      <c r="D2" s="94">
         <v>0.36</v>
       </c>
-      <c r="E2" s="92"/>
+      <c r="E2" s="96"/>
     </row>
     <row r="3" spans="1:5" ht="16" customHeight="1">
       <c r="A3" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="90" t="s">
+      <c r="B3" s="94" t="s">
         <v>140</v>
       </c>
-      <c r="C3" s="91"/>
-      <c r="D3" s="90">
+      <c r="C3" s="95"/>
+      <c r="D3" s="94">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="E3" s="92"/>
+      <c r="E3" s="96"/>
     </row>
     <row r="4" spans="1:5" ht="16" customHeight="1">
       <c r="A4" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="90">
+      <c r="B4" s="94">
         <v>0.5</v>
       </c>
-      <c r="C4" s="91"/>
-      <c r="D4" s="90">
+      <c r="C4" s="95"/>
+      <c r="D4" s="94">
         <v>0.35499999999999998</v>
       </c>
-      <c r="E4" s="92"/>
+      <c r="E4" s="96"/>
     </row>
     <row r="5" spans="1:5" ht="16" customHeight="1">
       <c r="A5" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="90" t="s">
+      <c r="B5" s="94" t="s">
         <v>140</v>
       </c>
-      <c r="C5" s="91"/>
-      <c r="D5" s="90">
+      <c r="C5" s="95"/>
+      <c r="D5" s="94">
         <v>4.5000000000000012E-2</v>
       </c>
-      <c r="E5" s="92"/>
+      <c r="E5" s="96"/>
     </row>
     <row r="6" spans="1:5" ht="16" customHeight="1">
       <c r="A6" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="90" t="s">
+      <c r="B6" s="94" t="s">
         <v>140</v>
       </c>
-      <c r="C6" s="91"/>
-      <c r="D6" s="90">
+      <c r="C6" s="95"/>
+      <c r="D6" s="94">
         <v>0.12</v>
       </c>
-      <c r="E6" s="92"/>
+      <c r="E6" s="96"/>
     </row>
     <row r="7" spans="1:5" ht="16" customHeight="1">
       <c r="A7" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="90" t="s">
+      <c r="B7" s="94" t="s">
         <v>140</v>
       </c>
-      <c r="C7" s="91"/>
-      <c r="D7" s="90">
+      <c r="C7" s="95"/>
+      <c r="D7" s="94">
         <v>7.5000000000000011E-2</v>
       </c>
-      <c r="E7" s="92"/>
+      <c r="E7" s="96"/>
     </row>
     <row r="8" spans="1:5" ht="16" customHeight="1">
       <c r="A8" s="68" t="s">
         <v>151</v>
       </c>
-      <c r="B8" s="93">
+      <c r="B8" s="97">
         <v>5.3832602562404443E-2</v>
       </c>
-      <c r="C8" s="94"/>
-      <c r="D8" s="93">
+      <c r="C8" s="98"/>
+      <c r="D8" s="97">
         <v>6.4431104932666197E-2</v>
       </c>
-      <c r="E8" s="95"/>
+      <c r="E8" s="99"/>
     </row>
     <row r="9" spans="1:5" ht="16" customHeight="1">
       <c r="A9" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="96">
+      <c r="B9" s="100">
         <v>0.39013325979698232</v>
       </c>
-      <c r="C9" s="91"/>
-      <c r="D9" s="96">
+      <c r="C9" s="95"/>
+      <c r="D9" s="100">
         <v>0.52364381017028427</v>
       </c>
-      <c r="E9" s="92"/>
+      <c r="E9" s="96"/>
     </row>
     <row r="10" spans="1:5" ht="16" customHeight="1">
       <c r="A10" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="90">
+      <c r="B10" s="94">
         <v>7.3904497600149111E-2</v>
       </c>
-      <c r="C10" s="91"/>
-      <c r="D10" s="90">
+      <c r="C10" s="95"/>
+      <c r="D10" s="94">
         <v>7.5095139422881152E-2</v>
       </c>
-      <c r="E10" s="92"/>
+      <c r="E10" s="96"/>
     </row>
     <row r="11" spans="1:5" ht="16" customHeight="1">
       <c r="A11" s="84" t="s">
@@ -23458,18 +23496,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:E6"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="B7:C7"/>
@@ -23478,6 +23504,18 @@
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D9:E9"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="B13:E21">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">

</xml_diff>